<commit_message>
feat(wishbone-bus): cascade child fabrics with SlaveBus
Allow one BusDef to be generated once and hung N times as Region windows
under a parent decoder, so parallel channels share RTL while the CPU still
reaches them. Demo splits SD/DMA/SHA256 into two sd_sha channels.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/demo/soc/fw/gen/wishbone/wishbone.xlsx
+++ b/demo/soc/fw/gen/wishbone/wishbone.xlsx
@@ -6,14 +6,15 @@
   <sheets>
     <sheet sheetId="1" name="sha256" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="smoke" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="MAP_soc_wb" state="visible" r:id="rId6"/>
+    <sheet sheetId="3" name="MAP_sd_sha" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="MAP_soc_wb" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="193">
   <si>
     <t xml:space="preserve">Sub-Addr
 (Hex)</t>
@@ -430,97 +431,124 @@
     <t>Description</t>
   </si>
   <si>
-    <t>sha256_0</t>
-  </si>
-  <si>
-    <t>0x03004000</t>
+    <t>sha256</t>
+  </si>
+  <si>
+    <t>0x00000040</t>
   </si>
   <si>
     <t>0xffffffc0</t>
   </si>
   <si>
-    <t>sha256</t>
-  </si>
-  <si>
     <t>0x00000000</t>
   </si>
   <si>
     <t>0x00000004</t>
   </si>
   <si>
-    <t>0x03004004</t>
+    <t>0x00000044</t>
   </si>
   <si>
     <t>0x00000008</t>
   </si>
   <si>
-    <t>0x03004008</t>
+    <t>0x00000048</t>
   </si>
   <si>
     <t>0x0000000c</t>
   </si>
   <si>
-    <t>0x0300400c</t>
+    <t>0x0000004c</t>
   </si>
   <si>
     <t>0x00000010</t>
   </si>
   <si>
-    <t>0x03004010</t>
+    <t>0x00000050</t>
   </si>
   <si>
     <t>0x00000014</t>
   </si>
   <si>
-    <t>0x03004014</t>
+    <t>0x00000054</t>
   </si>
   <si>
     <t>0x00000018</t>
   </si>
   <si>
-    <t>0x03004018</t>
+    <t>0x00000058</t>
   </si>
   <si>
     <t>0x0000001c</t>
   </si>
   <si>
-    <t>0x0300401c</t>
+    <t>0x0000005c</t>
   </si>
   <si>
     <t>0x00000020</t>
   </si>
   <si>
-    <t>0x03004020</t>
-  </si>
-  <si>
-    <t>sha256_1</t>
-  </si>
-  <si>
-    <t>0x03005000</t>
-  </si>
-  <si>
-    <t>0x03005004</t>
-  </si>
-  <si>
-    <t>0x03005008</t>
-  </si>
-  <si>
-    <t>0x0300500c</t>
-  </si>
-  <si>
-    <t>0x03005010</t>
-  </si>
-  <si>
-    <t>0x03005014</t>
-  </si>
-  <si>
-    <t>0x03005018</t>
-  </si>
-  <si>
-    <t>0x0300501c</t>
-  </si>
-  <si>
-    <t>0x03005020</t>
+    <t>0x00000060</t>
+  </si>
+  <si>
+    <t>ch0_sha256</t>
+  </si>
+  <si>
+    <t>0x03000040</t>
+  </si>
+  <si>
+    <t>0x03000044</t>
+  </si>
+  <si>
+    <t>0x03000048</t>
+  </si>
+  <si>
+    <t>0x0300004c</t>
+  </si>
+  <si>
+    <t>0x03000050</t>
+  </si>
+  <si>
+    <t>0x03000054</t>
+  </si>
+  <si>
+    <t>0x03000058</t>
+  </si>
+  <si>
+    <t>0x0300005c</t>
+  </si>
+  <si>
+    <t>0x03000060</t>
+  </si>
+  <si>
+    <t>ch1_sha256</t>
+  </si>
+  <si>
+    <t>0x03001040</t>
+  </si>
+  <si>
+    <t>0x03001044</t>
+  </si>
+  <si>
+    <t>0x03001048</t>
+  </si>
+  <si>
+    <t>0x0300104c</t>
+  </si>
+  <si>
+    <t>0x03001050</t>
+  </si>
+  <si>
+    <t>0x03001054</t>
+  </si>
+  <si>
+    <t>0x03001058</t>
+  </si>
+  <si>
+    <t>0x0300105c</t>
+  </si>
+  <si>
+    <t>0x03001060</t>
   </si>
   <si>
     <t>smoke</t>
@@ -3464,6 +3492,373 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="11" max="11" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="5">
+        <v>2</v>
+      </c>
+      <c r="E2" s="5">
+        <v>0</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D3" s="5">
+        <v>2</v>
+      </c>
+      <c r="E3" s="5">
+        <v>0</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="5">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D5" s="5">
+        <v>2</v>
+      </c>
+      <c r="E5" s="5">
+        <v>0</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D6" s="5">
+        <v>2</v>
+      </c>
+      <c r="E6" s="5">
+        <v>0</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D7" s="5">
+        <v>2</v>
+      </c>
+      <c r="E7" s="5">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D8" s="5">
+        <v>2</v>
+      </c>
+      <c r="E8" s="5">
+        <v>0</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D9" s="5">
+        <v>2</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D10" s="5">
+        <v>2</v>
+      </c>
+      <c r="E10" s="5">
+        <v>0</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -3510,10 +3905,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>137</v>
@@ -3528,13 +3923,13 @@
         <v>14</v>
       </c>
       <c r="G2" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H2" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="H2" s="5" t="s">
-        <v>139</v>
-      </c>
       <c r="I2" s="5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>13</v>
@@ -3545,10 +3940,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>137</v>
@@ -3563,13 +3958,13 @@
         <v>30</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>13</v>
@@ -3580,10 +3975,10 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>137</v>
@@ -3598,13 +3993,13 @@
         <v>34</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>13</v>
@@ -3615,10 +4010,10 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>137</v>
@@ -3633,13 +4028,13 @@
         <v>38</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>13</v>
@@ -3650,10 +4045,10 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>137</v>
@@ -3668,13 +4063,13 @@
         <v>42</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>13</v>
@@ -3685,10 +4080,10 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>137</v>
@@ -3703,13 +4098,13 @@
         <v>46</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>13</v>
@@ -3720,10 +4115,10 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>137</v>
@@ -3738,13 +4133,13 @@
         <v>50</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>13</v>
@@ -3755,10 +4150,10 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>137</v>
@@ -3773,13 +4168,13 @@
         <v>54</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>13</v>
@@ -3790,10 +4185,10 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>137</v>
@@ -3808,13 +4203,13 @@
         <v>58</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>13</v>
@@ -3825,16 +4220,16 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D11" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E11" s="5">
         <v>0</v>
@@ -3843,13 +4238,13 @@
         <v>14</v>
       </c>
       <c r="G11" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H11" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="H11" s="5" t="s">
-        <v>139</v>
-      </c>
       <c r="I11" s="5" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>13</v>
@@ -3860,16 +4255,16 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D12" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E12" s="5">
         <v>0</v>
@@ -3878,13 +4273,13 @@
         <v>30</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="J12" s="5" t="s">
         <v>13</v>
@@ -3895,16 +4290,16 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D13" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E13" s="5">
         <v>0</v>
@@ -3913,13 +4308,13 @@
         <v>34</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="J13" s="5" t="s">
         <v>13</v>
@@ -3930,16 +4325,16 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D14" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E14" s="5">
         <v>0</v>
@@ -3948,13 +4343,13 @@
         <v>38</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="J14" s="5" t="s">
         <v>13</v>
@@ -3965,16 +4360,16 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D15" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E15" s="5">
         <v>0</v>
@@ -3983,13 +4378,13 @@
         <v>42</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="J15" s="5" t="s">
         <v>13</v>
@@ -4000,16 +4395,16 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D16" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E16" s="5">
         <v>0</v>
@@ -4018,13 +4413,13 @@
         <v>46</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="J16" s="5" t="s">
         <v>13</v>
@@ -4035,16 +4430,16 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D17" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E17" s="5">
         <v>0</v>
@@ -4053,13 +4448,13 @@
         <v>50</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>13</v>
@@ -4070,16 +4465,16 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D18" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E18" s="5">
         <v>0</v>
@@ -4088,13 +4483,13 @@
         <v>54</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="J18" s="5" t="s">
         <v>13</v>
@@ -4105,16 +4500,16 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D19" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E19" s="5">
         <v>0</v>
@@ -4123,13 +4518,13 @@
         <v>58</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="J19" s="5" t="s">
         <v>13</v>
@@ -4140,10 +4535,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>137</v>
@@ -4158,13 +4553,13 @@
         <v>61</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="J20" s="5" t="s">
         <v>13</v>
@@ -4175,10 +4570,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>137</v>
@@ -4193,13 +4588,13 @@
         <v>68</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="J21" s="5" t="s">
         <v>13</v>
@@ -4210,10 +4605,10 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>137</v>
@@ -4228,13 +4623,13 @@
         <v>73</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="J22" s="5" t="s">
         <v>13</v>
@@ -4245,10 +4640,10 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>137</v>
@@ -4263,13 +4658,13 @@
         <v>79</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>13</v>
@@ -4280,10 +4675,10 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>137</v>
@@ -4298,13 +4693,13 @@
         <v>84</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="J24" s="5" t="s">
         <v>13</v>
@@ -4315,10 +4710,10 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>137</v>
@@ -4333,13 +4728,13 @@
         <v>89</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="J25" s="5" t="s">
         <v>13</v>
@@ -4350,10 +4745,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>137</v>
@@ -4368,13 +4763,13 @@
         <v>93</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="J26" s="5" t="s">
         <v>13</v>
@@ -4385,10 +4780,10 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>137</v>
@@ -4403,13 +4798,13 @@
         <v>98</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="J27" s="5" t="s">
         <v>100</v>
@@ -4420,10 +4815,10 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>137</v>
@@ -4438,13 +4833,13 @@
         <v>104</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="J28" s="5" t="s">
         <v>13</v>
@@ -4455,10 +4850,10 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>137</v>
@@ -4473,13 +4868,13 @@
         <v>109</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="J29" s="5" t="s">
         <v>13</v>
@@ -4490,10 +4885,10 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>137</v>
@@ -4508,13 +4903,13 @@
         <v>113</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="J30" s="5" t="s">
         <v>13</v>
@@ -4525,10 +4920,10 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>137</v>
@@ -4543,13 +4938,13 @@
         <v>117</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="J31" s="5" t="s">
         <v>13</v>
@@ -4560,10 +4955,10 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>137</v>
@@ -4578,13 +4973,13 @@
         <v>121</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="J32" s="5" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
feat(wishbone-regfile): Excel-only long notes beside desc
Keep desc a one-line summary for RTL, C, and uvm_reg. Field notes continue the same Description cell after a newline; a regfile note hangs on the header comment so bit-width formulas stay aligned.
</commit_message>
<xml_diff>
--- a/demo/soc/fw/gen/wishbone/wishbone.xlsx
+++ b/demo/soc/fw/gen/wishbone/wishbone.xlsx
@@ -13,6 +13,27 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">SHA256 CSR (CTRL + HASH0..7); instantiate once per fabric lane
+CTRL is the only SW/HW handshake cell. Glue holds the core in reset
+while soft_reset stays 1; software must write 0 before the next message.
+HASH0..7 are digest words. Each 32-bit word is byte-reversed versus
+the on-wire SHA-256 digest.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="193">
   <si>
@@ -101,7 +122,9 @@
     <t>done_clear</t>
   </si>
   <si>
-    <t>Write 1 → pulse; glue clears sticky done</t>
+    <t xml:space="preserve">Write 1 → pulse; glue clears sticky done
+Pulse only. The stored bit reads back 0.
+Glue clears sticky done on this write; it does not touch HASH*.</t>
   </si>
   <si>
     <t>RW</t>
@@ -110,7 +133,9 @@
     <t>soft_reset</t>
   </si>
   <si>
-    <t>Soft reset hash core</t>
+    <t xml:space="preserve">Soft reset hash core
+Write 1 to reset the core. Glue holds reset while this bit stays 1.
+Software must write 0 before starting the next message.</t>
   </si>
   <si>
     <t>00000004</t>
@@ -1950,6 +1975,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3501,7 +3527,7 @@
     <col min="11" max="11" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>124</v>
       </c>
@@ -3868,7 +3894,7 @@
     <col min="11" max="11" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>124</v>
       </c>

</xml_diff>

<commit_message>
feat(wishbone): split address tag from working-bank mux
TagFromAddr selects the accessed bank. i_<domain>_mux_sel, driven by BANKSEL, selects the sideband copy, and ACTIVE reads that copy back. JTAG covers both paths after firmware pass.
</commit_message>
<xml_diff>
--- a/demo/soc/fw/gen/wishbone/wishbone.xlsx
+++ b/demo/soc/fw/gen/wishbone/wishbone.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="200">
   <si>
     <t xml:space="preserve">Sub-Addr
 (Hex)</t>
@@ -366,13 +366,28 @@
     <t>BANKSEL</t>
   </si>
   <si>
-    <t>Shadow bank select (drives fabric TGA)</t>
+    <t>Saved working bank</t>
   </si>
   <si>
     <t>bank_sel</t>
   </si>
   <si>
-    <t>Shadow bank for WB accesses</t>
+    <t>Working bank</t>
+  </si>
+  <si>
+    <t>00000034</t>
+  </si>
+  <si>
+    <t>ACTIVE</t>
+  </si>
+  <si>
+    <t>Muxed working cfg</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>Working copy of BANK.cfg</t>
   </si>
   <si>
     <t>00000030</t>
@@ -607,6 +622,12 @@
   </si>
   <si>
     <t>0x0300602c</t>
+  </si>
+  <si>
+    <t>0x00000034</t>
+  </si>
+  <si>
+    <t>0x03006034</t>
   </si>
   <si>
     <t>0x00000030</t>
@@ -1981,7 +2002,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="5" max="5" width="16" customWidth="1"/>
@@ -3211,7 +3232,7 @@
         <v>13</v>
       </c>
       <c r="B33" s="3">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C33" s="3">
         <v>31</v>
@@ -3252,7 +3273,7 @@
         <v>0</v>
       </c>
       <c r="C34" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D34" s="4">
         <f>C34-B34+1</f>
@@ -3261,7 +3282,7 @@
         <f>CONCATENATE(D34,"'h",J34)</f>
       </c>
       <c r="F34" s="4" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="G34" s="4" t="s">
         <v>111</v>
@@ -3284,7 +3305,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>57</v>
+        <v>113</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>13</v>
@@ -3293,7 +3314,7 @@
         <v>13</v>
       </c>
       <c r="D35" s="2">
-        <f>SUM(D36:D36)</f>
+        <f>SUM(D36:D37)</f>
       </c>
       <c r="E35" s="2">
         <f>CONCATENATE("32'h",J35)</f>
@@ -3302,10 +3323,10 @@
         <v>13</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>13</v>
@@ -3314,199 +3335,313 @@
         <f>LOWER(DEC2HEX(K35, 8))</f>
       </c>
       <c r="K35" s="2">
-        <f>SUM(K36:K36)</f>
+        <f>SUM(K36:K37)</f>
       </c>
       <c r="L35" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B36" s="4">
-        <v>0</v>
-      </c>
-      <c r="C36" s="4">
+      <c r="A36" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36" s="3">
+        <v>1</v>
+      </c>
+      <c r="C36" s="3">
         <v>31</v>
       </c>
-      <c r="D36" s="4">
+      <c r="D36" s="3">
         <f>C36-B36+1</f>
       </c>
-      <c r="E36" s="4">
+      <c r="E36" s="3">
         <f>CONCATENATE(D36,"'h",J36)</f>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="F36" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="3">
+        <v>0</v>
+      </c>
+      <c r="J36" s="3">
+        <f>LOWER(DEC2HEX((I36)))</f>
+      </c>
+      <c r="K36" s="3">
+        <f>I36*(2^B36)</f>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="4">
+        <v>0</v>
+      </c>
+      <c r="C37" s="4">
+        <v>0</v>
+      </c>
+      <c r="D37" s="4">
+        <f>C37-B37+1</f>
+      </c>
+      <c r="E37" s="4">
+        <f>CONCATENATE(D37,"'h",J37)</f>
+      </c>
+      <c r="F37" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G36" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="H36" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="I36" s="4">
-        <v>0</v>
-      </c>
-      <c r="J36" s="4">
-        <f>LOWER(DEC2HEX((I36)))</f>
-      </c>
-      <c r="K36" s="4">
-        <f>I36*(2^B36)</f>
-      </c>
-      <c r="L36" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
+      <c r="G37" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D37" s="2">
-        <f>SUM(D38:D38)</f>
-      </c>
-      <c r="E37" s="2">
-        <f>CONCATENATE("32'h",J37)</f>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G37" s="2" t="s">
+      <c r="H37" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="I37" s="4">
+        <v>0</v>
+      </c>
+      <c r="J37" s="4">
+        <f>LOWER(DEC2HEX((I37)))</f>
+      </c>
+      <c r="K37" s="4">
+        <f>I37*(2^B37)</f>
+      </c>
+      <c r="L37" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="2">
+        <f>SUM(D39:D39)</f>
+      </c>
+      <c r="E38" s="2">
+        <f>CONCATENATE("32'h",J38)</f>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="I37" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J37" s="2">
-        <f>LOWER(DEC2HEX(K37, 8))</f>
-      </c>
-      <c r="K37" s="2">
-        <f>SUM(K38:K38)</f>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B38" s="4">
-        <v>0</v>
-      </c>
-      <c r="C38" s="4">
+      <c r="H38" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J38" s="2">
+        <f>LOWER(DEC2HEX(K38, 8))</f>
+      </c>
+      <c r="K38" s="2">
+        <f>SUM(K39:K39)</f>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B39" s="4">
+        <v>0</v>
+      </c>
+      <c r="C39" s="4">
         <v>31</v>
       </c>
-      <c r="D38" s="4">
-        <f>C38-B38+1</f>
-      </c>
-      <c r="E38" s="4">
-        <f>CONCATENATE(D38,"'h",J38)</f>
-      </c>
-      <c r="F38" s="4" t="s">
+      <c r="D39" s="4">
+        <f>C39-B39+1</f>
+      </c>
+      <c r="E39" s="4">
+        <f>CONCATENATE(D39,"'h",J39)</f>
+      </c>
+      <c r="F39" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G38" s="4" t="s">
+      <c r="G39" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="H39" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="H38" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="I38" s="4">
-        <v>0</v>
-      </c>
-      <c r="J38" s="4">
-        <f>LOWER(DEC2HEX((I38)))</f>
-      </c>
-      <c r="K38" s="4">
-        <f>I38*(2^B38)</f>
-      </c>
-      <c r="L38" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D39" s="2">
-        <f>SUM(D40:D40)</f>
-      </c>
-      <c r="E39" s="2">
-        <f>CONCATENATE("32'h",J39)</f>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G39" s="2" t="s">
+      <c r="I39" s="4">
+        <v>0</v>
+      </c>
+      <c r="J39" s="4">
+        <f>LOWER(DEC2HEX((I39)))</f>
+      </c>
+      <c r="K39" s="4">
+        <f>I39*(2^B39)</f>
+      </c>
+      <c r="L39" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="H39" s="2" t="s">
+      <c r="B40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" s="2">
+        <f>SUM(D41:D41)</f>
+      </c>
+      <c r="E40" s="2">
+        <f>CONCATENATE("32'h",J40)</f>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="I39" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J39" s="2">
-        <f>LOWER(DEC2HEX(K39, 8))</f>
-      </c>
-      <c r="K39" s="2">
-        <f>SUM(K40:K40)</f>
-      </c>
-      <c r="L39" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B40" s="4">
-        <v>0</v>
-      </c>
-      <c r="C40" s="4">
+      <c r="H40" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J40" s="2">
+        <f>LOWER(DEC2HEX(K40, 8))</f>
+      </c>
+      <c r="K40" s="2">
+        <f>SUM(K41:K41)</f>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" s="4">
+        <v>0</v>
+      </c>
+      <c r="C41" s="4">
         <v>31</v>
       </c>
-      <c r="D40" s="4">
-        <f>C40-B40+1</f>
-      </c>
-      <c r="E40" s="4">
-        <f>CONCATENATE(D40,"'h",J40)</f>
-      </c>
-      <c r="F40" s="4" t="s">
+      <c r="D41" s="4">
+        <f>C41-B41+1</f>
+      </c>
+      <c r="E41" s="4">
+        <f>CONCATENATE(D41,"'h",J41)</f>
+      </c>
+      <c r="F41" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="G41" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="H41" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="H40" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="I40" s="4">
-        <v>0</v>
-      </c>
-      <c r="J40" s="4">
-        <f>LOWER(DEC2HEX((I40)))</f>
-      </c>
-      <c r="K40" s="4">
-        <f>I40*(2^B40)</f>
-      </c>
-      <c r="L40" s="4" t="s">
+      <c r="I41" s="4">
+        <v>0</v>
+      </c>
+      <c r="J41" s="4">
+        <f>LOWER(DEC2HEX((I41)))</f>
+      </c>
+      <c r="K41" s="4">
+        <f>I41*(2^B41)</f>
+      </c>
+      <c r="L41" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" s="2">
+        <f>SUM(D43:D43)</f>
+      </c>
+      <c r="E42" s="2">
+        <f>CONCATENATE("32'h",J42)</f>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J42" s="2">
+        <f>LOWER(DEC2HEX(K42, 8))</f>
+      </c>
+      <c r="K42" s="2">
+        <f>SUM(K43:K43)</f>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A43" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B43" s="4">
+        <v>0</v>
+      </c>
+      <c r="C43" s="4">
+        <v>31</v>
+      </c>
+      <c r="D43" s="4">
+        <f>C43-B43+1</f>
+      </c>
+      <c r="E43" s="4">
+        <f>CONCATENATE(D43,"'h",J43)</f>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="I43" s="4">
+        <v>0</v>
+      </c>
+      <c r="J43" s="4">
+        <f>LOWER(DEC2HEX((I43)))</f>
+      </c>
+      <c r="K43" s="4">
+        <f>I43*(2^B43)</f>
+      </c>
+      <c r="L43" s="4" t="s">
         <v>13</v>
       </c>
     </row>
@@ -3529,48 +3664,48 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D2" s="5">
         <v>2</v>
@@ -3582,13 +3717,13 @@
         <v>14</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>13</v>
@@ -3599,13 +3734,13 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D3" s="5">
         <v>2</v>
@@ -3617,13 +3752,13 @@
         <v>30</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>13</v>
@@ -3634,13 +3769,13 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D4" s="5">
         <v>2</v>
@@ -3652,13 +3787,13 @@
         <v>34</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>13</v>
@@ -3669,13 +3804,13 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D5" s="5">
         <v>2</v>
@@ -3687,13 +3822,13 @@
         <v>38</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>13</v>
@@ -3704,13 +3839,13 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D6" s="5">
         <v>2</v>
@@ -3722,13 +3857,13 @@
         <v>42</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>13</v>
@@ -3739,13 +3874,13 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D7" s="5">
         <v>2</v>
@@ -3757,13 +3892,13 @@
         <v>46</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>13</v>
@@ -3774,13 +3909,13 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D8" s="5">
         <v>2</v>
@@ -3792,13 +3927,13 @@
         <v>50</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>13</v>
@@ -3809,13 +3944,13 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D9" s="5">
         <v>2</v>
@@ -3827,13 +3962,13 @@
         <v>54</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>13</v>
@@ -3844,13 +3979,13 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D10" s="5">
         <v>2</v>
@@ -3862,13 +3997,13 @@
         <v>58</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>13</v>
@@ -3885,7 +4020,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -3896,48 +4031,48 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D2" s="5">
         <v>2</v>
@@ -3949,13 +4084,13 @@
         <v>14</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>13</v>
@@ -3966,13 +4101,13 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D3" s="5">
         <v>2</v>
@@ -3984,13 +4119,13 @@
         <v>30</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>13</v>
@@ -4001,13 +4136,13 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D4" s="5">
         <v>2</v>
@@ -4019,13 +4154,13 @@
         <v>34</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>13</v>
@@ -4036,13 +4171,13 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D5" s="5">
         <v>2</v>
@@ -4054,13 +4189,13 @@
         <v>38</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>13</v>
@@ -4071,13 +4206,13 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D6" s="5">
         <v>2</v>
@@ -4089,13 +4224,13 @@
         <v>42</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>13</v>
@@ -4106,13 +4241,13 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D7" s="5">
         <v>2</v>
@@ -4124,13 +4259,13 @@
         <v>46</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>13</v>
@@ -4141,13 +4276,13 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D8" s="5">
         <v>2</v>
@@ -4159,13 +4294,13 @@
         <v>50</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>13</v>
@@ -4176,13 +4311,13 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D9" s="5">
         <v>2</v>
@@ -4194,13 +4329,13 @@
         <v>54</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>13</v>
@@ -4211,13 +4346,13 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D10" s="5">
         <v>2</v>
@@ -4229,13 +4364,13 @@
         <v>58</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>13</v>
@@ -4246,13 +4381,13 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D11" s="5">
         <v>2</v>
@@ -4264,13 +4399,13 @@
         <v>14</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>13</v>
@@ -4281,13 +4416,13 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D12" s="5">
         <v>2</v>
@@ -4299,13 +4434,13 @@
         <v>30</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="J12" s="5" t="s">
         <v>13</v>
@@ -4316,13 +4451,13 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D13" s="5">
         <v>2</v>
@@ -4334,13 +4469,13 @@
         <v>34</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="J13" s="5" t="s">
         <v>13</v>
@@ -4351,13 +4486,13 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D14" s="5">
         <v>2</v>
@@ -4369,13 +4504,13 @@
         <v>38</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="J14" s="5" t="s">
         <v>13</v>
@@ -4386,13 +4521,13 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D15" s="5">
         <v>2</v>
@@ -4404,13 +4539,13 @@
         <v>42</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="J15" s="5" t="s">
         <v>13</v>
@@ -4421,13 +4556,13 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D16" s="5">
         <v>2</v>
@@ -4439,13 +4574,13 @@
         <v>46</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="J16" s="5" t="s">
         <v>13</v>
@@ -4456,13 +4591,13 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D17" s="5">
         <v>2</v>
@@ -4474,13 +4609,13 @@
         <v>50</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>13</v>
@@ -4491,13 +4626,13 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D18" s="5">
         <v>2</v>
@@ -4509,13 +4644,13 @@
         <v>54</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="J18" s="5" t="s">
         <v>13</v>
@@ -4526,13 +4661,13 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D19" s="5">
         <v>2</v>
@@ -4544,13 +4679,13 @@
         <v>58</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="J19" s="5" t="s">
         <v>13</v>
@@ -4561,13 +4696,13 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D20" s="5">
         <v>3</v>
@@ -4579,13 +4714,13 @@
         <v>61</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="J20" s="5" t="s">
         <v>13</v>
@@ -4596,13 +4731,13 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D21" s="5">
         <v>3</v>
@@ -4614,13 +4749,13 @@
         <v>68</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="J21" s="5" t="s">
         <v>13</v>
@@ -4631,13 +4766,13 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D22" s="5">
         <v>3</v>
@@ -4649,13 +4784,13 @@
         <v>73</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="J22" s="5" t="s">
         <v>13</v>
@@ -4666,13 +4801,13 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D23" s="5">
         <v>3</v>
@@ -4684,13 +4819,13 @@
         <v>79</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>13</v>
@@ -4701,13 +4836,13 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D24" s="5">
         <v>3</v>
@@ -4719,13 +4854,13 @@
         <v>84</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="J24" s="5" t="s">
         <v>13</v>
@@ -4736,13 +4871,13 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D25" s="5">
         <v>3</v>
@@ -4754,13 +4889,13 @@
         <v>89</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="J25" s="5" t="s">
         <v>13</v>
@@ -4771,13 +4906,13 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D26" s="5">
         <v>3</v>
@@ -4789,13 +4924,13 @@
         <v>93</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="J26" s="5" t="s">
         <v>13</v>
@@ -4806,13 +4941,13 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D27" s="5">
         <v>3</v>
@@ -4824,13 +4959,13 @@
         <v>98</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="J27" s="5" t="s">
         <v>100</v>
@@ -4841,13 +4976,13 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D28" s="5">
         <v>3</v>
@@ -4859,13 +4994,13 @@
         <v>104</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="J28" s="5" t="s">
         <v>13</v>
@@ -4876,13 +5011,13 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D29" s="5">
         <v>3</v>
@@ -4894,13 +5029,13 @@
         <v>109</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="J29" s="5" t="s">
         <v>13</v>
@@ -4911,13 +5046,13 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D30" s="5">
         <v>3</v>
@@ -4926,33 +5061,33 @@
         <v>2</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>153</v>
+        <v>193</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="J30" s="5" t="s">
         <v>13</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D31" s="5">
         <v>3</v>
@@ -4961,33 +5096,33 @@
         <v>2</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>189</v>
+        <v>158</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="J31" s="5" t="s">
         <v>13</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D32" s="5">
         <v>3</v>
@@ -4996,22 +5131,57 @@
         <v>2</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="J32" s="5" t="s">
         <v>13</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D33" s="5">
+        <v>3</v>
+      </c>
+      <c r="E33" s="5">
+        <v>2</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(wishbone): print bus trees and pack docs into the release
Generation prints a colored address tree and each regfile file as it is written. Excel lists one row per address leaf, with independent buses on separate sheets. The release script gzips docs and every demo; docs unpack writes them out.
</commit_message>
<xml_diff>
--- a/demo/soc/fw/gen/wishbone/wishbone.xlsx
+++ b/demo/soc/fw/gen/wishbone/wishbone.xlsx
@@ -6,8 +6,7 @@
   <sheets>
     <sheet sheetId="1" name="sha256" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="smoke" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="MAP_sd_sha" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="MAP_soc_wb" state="visible" r:id="rId7"/>
+    <sheet sheetId="3" name="soc_wb" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="178">
   <si>
     <t xml:space="preserve">Sub-Addr
 (Hex)</t>
@@ -438,31 +437,22 @@
     <t>key_2</t>
   </si>
   <si>
-    <t>Slave</t>
-  </si>
-  <si>
-    <t>Base</t>
-  </si>
-  <si>
-    <t>Mask</t>
-  </si>
-  <si>
-    <t>Pipe</t>
-  </si>
-  <si>
-    <t>Tag</t>
-  </si>
-  <si>
-    <t>Cell</t>
-  </si>
-  <si>
-    <t>Sheet</t>
-  </si>
-  <si>
-    <t>Offset</t>
-  </si>
-  <si>
-    <t>Absolute</t>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Window</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Leaf</t>
+  </si>
+  <si>
+    <t>Bits</t>
+  </si>
+  <si>
+    <t>Broadcast</t>
   </si>
   <si>
     <t>Shadow</t>
@@ -471,184 +461,127 @@
     <t>Description</t>
   </si>
   <si>
+    <t>0x00000000</t>
+  </si>
+  <si>
+    <t>sram</t>
+  </si>
+  <si>
+    <t>0x00010000</t>
+  </si>
+  <si>
+    <t>64 KiB SRAM</t>
+  </si>
+  <si>
+    <t>0x01000000</t>
+  </si>
+  <si>
+    <t>flash_xip</t>
+  </si>
+  <si>
+    <t>SPI flash XIP</t>
+  </si>
+  <si>
+    <t>0x02000000</t>
+  </si>
+  <si>
+    <t>flash_cfg</t>
+  </si>
+  <si>
+    <t>0x00000004</t>
+  </si>
+  <si>
+    <t>SPI flash cfg</t>
+  </si>
+  <si>
+    <t>0x02000004</t>
+  </si>
+  <si>
+    <t>uart</t>
+  </si>
+  <si>
+    <t>0x00000008</t>
+  </si>
+  <si>
+    <t>simpleuart</t>
+  </si>
+  <si>
+    <t>0x02000010</t>
+  </si>
+  <si>
+    <t>testout</t>
+  </si>
+  <si>
+    <t>test output</t>
+  </si>
+  <si>
+    <t>0x03000000</t>
+  </si>
+  <si>
+    <t>ch0</t>
+  </si>
+  <si>
+    <t>0x00001000</t>
+  </si>
+  <si>
+    <t>sd_sha</t>
+  </si>
+  <si>
+    <t>SD + DMA + SHA256 channel interconnect (uplink + engine)</t>
+  </si>
+  <si>
+    <t>sd</t>
+  </si>
+  <si>
+    <t>0x00000010</t>
+  </si>
+  <si>
+    <t>sdspi CSR</t>
+  </si>
+  <si>
+    <t>0x03000010</t>
+  </si>
+  <si>
+    <t>dma</t>
+  </si>
+  <si>
+    <t>sd_rd_dma CSR</t>
+  </si>
+  <si>
+    <t>0x03000040</t>
+  </si>
+  <si>
     <t>sha256</t>
   </si>
   <si>
-    <t>0x00000040</t>
-  </si>
-  <si>
-    <t>0xffffffc0</t>
-  </si>
-  <si>
-    <t>0x00000000</t>
-  </si>
-  <si>
-    <t>0x00000004</t>
-  </si>
-  <si>
-    <t>0x00000044</t>
-  </si>
-  <si>
-    <t>0x00000008</t>
-  </si>
-  <si>
-    <t>0x00000048</t>
-  </si>
-  <si>
-    <t>0x0000000c</t>
-  </si>
-  <si>
-    <t>0x0000004c</t>
-  </si>
-  <si>
-    <t>0x00000010</t>
-  </si>
-  <si>
-    <t>0x00000050</t>
-  </si>
-  <si>
-    <t>0x00000014</t>
-  </si>
-  <si>
-    <t>0x00000054</t>
-  </si>
-  <si>
-    <t>0x00000018</t>
-  </si>
-  <si>
-    <t>0x00000058</t>
-  </si>
-  <si>
-    <t>0x0000001c</t>
-  </si>
-  <si>
-    <t>0x0000005c</t>
-  </si>
-  <si>
-    <t>0x00000020</t>
-  </si>
-  <si>
-    <t>0x00000060</t>
-  </si>
-  <si>
-    <t>ch0_sha256</t>
-  </si>
-  <si>
-    <t>0x03000040</t>
-  </si>
-  <si>
-    <t>0x03000044</t>
-  </si>
-  <si>
-    <t>0x03000048</t>
-  </si>
-  <si>
-    <t>0x0300004c</t>
-  </si>
-  <si>
-    <t>0x03000050</t>
-  </si>
-  <si>
-    <t>0x03000054</t>
-  </si>
-  <si>
-    <t>0x03000058</t>
-  </si>
-  <si>
-    <t>0x0300005c</t>
-  </si>
-  <si>
-    <t>0x03000060</t>
-  </si>
-  <si>
-    <t>ch1_sha256</t>
-  </si>
-  <si>
-    <t>0x03001040</t>
-  </si>
-  <si>
-    <t>0x03001044</t>
-  </si>
-  <si>
-    <t>0x03001048</t>
-  </si>
-  <si>
-    <t>0x0300104c</t>
-  </si>
-  <si>
-    <t>0x03001050</t>
-  </si>
-  <si>
-    <t>0x03001054</t>
-  </si>
-  <si>
-    <t>0x03001058</t>
-  </si>
-  <si>
-    <t>0x0300105c</t>
-  </si>
-  <si>
-    <t>0x03001060</t>
+    <t>0x00000024</t>
+  </si>
+  <si>
+    <t>CTRL@0x0 soft_reset[undefined:undefined] done_clear[undefined:undefined] busy[undefined:undefined] done[undefined:undefined]; HASH0@0x4 hash0[undefined:undefined]; HASH1@0x8 hash1[undefined:undefined]; HASH2@0xc hash2[undefined:undefined]; HASH3@0x10 hash3[undefined:undefined]; HASH4@0x14 hash4[undefined:undefined]; HASH5@0x18 hash5[undefined:undefined]; HASH6@0x1c hash6[undefined:undefined]; HASH7@0x20 hash7[undefined:undefined]</t>
+  </si>
+  <si>
+    <t>SHA256 CSR (CTRL + HASH0..7); instantiate once per fabric lane</t>
+  </si>
+  <si>
+    <t>0x03001000</t>
+  </si>
+  <si>
+    <t>ch1</t>
+  </si>
+  <si>
+    <t>0x03006000</t>
   </si>
   <si>
     <t>smoke</t>
   </si>
   <si>
-    <t>0x03006000</t>
-  </si>
-  <si>
-    <t>0x03006004</t>
-  </si>
-  <si>
-    <t>0x03006008</t>
-  </si>
-  <si>
-    <t>0x0300600c</t>
-  </si>
-  <si>
-    <t>0x03006010</t>
-  </si>
-  <si>
-    <t>0x03006014</t>
-  </si>
-  <si>
-    <t>0x03006018</t>
-  </si>
-  <si>
-    <t>0x0300601c</t>
-  </si>
-  <si>
-    <t>0x0000002c</t>
-  </si>
-  <si>
-    <t>0x0300602c</t>
-  </si>
-  <si>
-    <t>0x00000034</t>
-  </si>
-  <si>
-    <t>0x03006034</t>
-  </si>
-  <si>
-    <t>0x00000030</t>
-  </si>
-  <si>
-    <t>0x03006030</t>
-  </si>
-  <si>
-    <t>0x03006020</t>
-  </si>
-  <si>
-    <t>0x00000024</t>
-  </si>
-  <si>
-    <t>0x03006024</t>
-  </si>
-  <si>
-    <t>0x00000028</t>
-  </si>
-  <si>
-    <t>0x03006028</t>
+    <t>0x00000038</t>
+  </si>
+  <si>
+    <t>ID@0x0 magic[undefined:undefined] version[undefined:undefined]; STATUS@0x4 busy[undefined:undefined] code[undefined:undefined]; CFG@0x8 enable[undefined:undefined] mode[undefined:undefined]; FEED@0xc capture[undefined:undefined]; FIFO@0x10 data[undefined:undefined]; CMD@0x14 go[undefined:undefined]; IRQ@0x18 sticky[undefined:undefined]; BANK@0x1c cfg[undefined:undefined]; BANKSEL@0x2c bank_sel[undefined:undefined]; ACTIVE@0x34 value[undefined:undefined]; FABRIC@0x30 rb_grant_en[undefined:undefined]; key_key_0@0x20 key_0[undefined:undefined]; key_key_1@0x24 key_1[undefined:undefined]; key_key_2@0x28 key_2[undefined:undefined]</t>
+  </si>
+  <si>
+    <t>SoC regfile smoke bank (RC/RO/RW/RWW/RWE/W1P/W1C/shadow/wide)</t>
   </si>
 </sst>
 </file>
@@ -3653,16 +3586,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="11" max="11" width="40" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="48" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>129</v>
       </c>
@@ -3687,1501 +3620,291 @@
       <c r="H1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="B2" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="C2" s="5" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="D2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B2" s="5" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="B3" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="5">
-        <v>2</v>
-      </c>
-      <c r="E2" s="5">
-        <v>0</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H2" s="5" t="s">
+      <c r="C3" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D3" s="5">
-        <v>2</v>
-      </c>
-      <c r="E3" s="5">
-        <v>0</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H3" s="5" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="B4" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="J3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>141</v>
-      </c>
       <c r="C4" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D4" s="5">
-        <v>2</v>
-      </c>
-      <c r="E4" s="5">
-        <v>0</v>
+        <v>146</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>140</v>
+        <v>13</v>
       </c>
       <c r="H4" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="I4" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D5" s="5">
-        <v>2</v>
-      </c>
-      <c r="E5" s="5">
-        <v>0</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D6" s="5">
-        <v>2</v>
-      </c>
-      <c r="E6" s="5">
-        <v>0</v>
+      <c r="D6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>140</v>
+        <v>13</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D7" s="5">
-        <v>2</v>
-      </c>
-      <c r="E7" s="5">
-        <v>0</v>
+        <v>157</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>140</v>
+        <v>13</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D8" s="5">
-        <v>2</v>
-      </c>
-      <c r="E8" s="5">
-        <v>0</v>
+        <v>161</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>140</v>
+        <v>13</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D9" s="5">
-        <v>2</v>
-      </c>
-      <c r="E9" s="5">
-        <v>0</v>
+        <v>161</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>140</v>
+        <v>13</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="I9" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="J9" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D10" s="5">
-        <v>2</v>
-      </c>
-      <c r="E10" s="5">
-        <v>0</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H10" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="E11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="J10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K33"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="11" max="11" width="40" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D2" s="5">
-        <v>2</v>
-      </c>
-      <c r="E2" s="5">
-        <v>0</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D3" s="5">
-        <v>2</v>
-      </c>
-      <c r="E3" s="5">
-        <v>0</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D4" s="5">
-        <v>2</v>
-      </c>
-      <c r="E4" s="5">
-        <v>0</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D5" s="5">
-        <v>2</v>
-      </c>
-      <c r="E5" s="5">
-        <v>0</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D6" s="5">
-        <v>2</v>
-      </c>
-      <c r="E6" s="5">
-        <v>0</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D7" s="5">
-        <v>2</v>
-      </c>
-      <c r="E7" s="5">
-        <v>0</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D8" s="5">
-        <v>2</v>
-      </c>
-      <c r="E8" s="5">
-        <v>0</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D9" s="5">
-        <v>2</v>
-      </c>
-      <c r="E9" s="5">
-        <v>0</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D10" s="5">
-        <v>2</v>
-      </c>
-      <c r="E10" s="5">
-        <v>0</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D11" s="5">
-        <v>2</v>
-      </c>
-      <c r="E11" s="5">
-        <v>0</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K11" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D12" s="5">
-        <v>2</v>
-      </c>
-      <c r="E12" s="5">
-        <v>0</v>
+        <v>175</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>176</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D13" s="5">
-        <v>2</v>
-      </c>
-      <c r="E13" s="5">
-        <v>0</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="J13" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K13" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D14" s="5">
-        <v>2</v>
-      </c>
-      <c r="E14" s="5">
-        <v>0</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K14" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D15" s="5">
-        <v>2</v>
-      </c>
-      <c r="E15" s="5">
-        <v>0</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="J15" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K15" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D16" s="5">
-        <v>2</v>
-      </c>
-      <c r="E16" s="5">
-        <v>0</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K16" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D17" s="5">
-        <v>2</v>
-      </c>
-      <c r="E17" s="5">
-        <v>0</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="I17" s="5" t="s">
         <v>177</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K17" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D18" s="5">
-        <v>2</v>
-      </c>
-      <c r="E18" s="5">
-        <v>0</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K18" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D19" s="5">
-        <v>2</v>
-      </c>
-      <c r="E19" s="5">
-        <v>0</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K19" s="5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D20" s="5">
-        <v>3</v>
-      </c>
-      <c r="E20" s="5">
-        <v>2</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="I20" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="J20" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K20" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D21" s="5">
-        <v>3</v>
-      </c>
-      <c r="E21" s="5">
-        <v>2</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K21" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D22" s="5">
-        <v>3</v>
-      </c>
-      <c r="E22" s="5">
-        <v>2</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I22" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="J22" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K22" s="5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D23" s="5">
-        <v>3</v>
-      </c>
-      <c r="E23" s="5">
-        <v>2</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H23" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="J23" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K23" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D24" s="5">
-        <v>3</v>
-      </c>
-      <c r="E24" s="5">
-        <v>2</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="I24" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="J24" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K24" s="5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D25" s="5">
-        <v>3</v>
-      </c>
-      <c r="E25" s="5">
-        <v>2</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="I25" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D26" s="5">
-        <v>3</v>
-      </c>
-      <c r="E26" s="5">
-        <v>2</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K26" s="5" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D27" s="5">
-        <v>3</v>
-      </c>
-      <c r="E27" s="5">
-        <v>2</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="J27" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="K27" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D28" s="5">
-        <v>3</v>
-      </c>
-      <c r="E28" s="5">
-        <v>2</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="I28" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="J28" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K28" s="5" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D29" s="5">
-        <v>3</v>
-      </c>
-      <c r="E29" s="5">
-        <v>2</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="I29" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K29" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D30" s="5">
-        <v>3</v>
-      </c>
-      <c r="E30" s="5">
-        <v>2</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H30" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="I30" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="J30" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K30" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D31" s="5">
-        <v>3</v>
-      </c>
-      <c r="E31" s="5">
-        <v>2</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H31" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="I31" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="J31" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K31" s="5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D32" s="5">
-        <v>3</v>
-      </c>
-      <c r="E32" s="5">
-        <v>2</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H32" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="I32" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="J32" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K32" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D33" s="5">
-        <v>3</v>
-      </c>
-      <c r="E33" s="5">
-        <v>2</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="I33" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="J33" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K33" s="5" t="s">
-        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(wishbone): regenerate soc showcase xlsx
The committed workbook still carried the fixed emitter's bug output
(field bit ranges rendered as undefined:undefined). Content now matches
the current generator.
</commit_message>
<xml_diff>
--- a/demo/soc/fw/gen/wishbone/wishbone.xlsx
+++ b/demo/soc/fw/gen/wishbone/wishbone.xlsx
@@ -557,7 +557,7 @@
     <t>0x00000024</t>
   </si>
   <si>
-    <t>CTRL@0x0 soft_reset[undefined:undefined] done_clear[undefined:undefined] busy[undefined:undefined] done[undefined:undefined]; HASH0@0x4 hash0[undefined:undefined]; HASH1@0x8 hash1[undefined:undefined]; HASH2@0xc hash2[undefined:undefined]; HASH3@0x10 hash3[undefined:undefined]; HASH4@0x14 hash4[undefined:undefined]; HASH5@0x18 hash5[undefined:undefined]; HASH6@0x1c hash6[undefined:undefined]; HASH7@0x20 hash7[undefined:undefined]</t>
+    <t>CTRL@0x0 soft_reset[0:0] done_clear[1:1] busy[8:8] done[9:9]; HASH0@0x4 hash0[31:0]; HASH1@0x8 hash1[31:0]; HASH2@0xc hash2[31:0]; HASH3@0x10 hash3[31:0]; HASH4@0x14 hash4[31:0]; HASH5@0x18 hash5[31:0]; HASH6@0x1c hash6[31:0]; HASH7@0x20 hash7[31:0]</t>
   </si>
   <si>
     <t>SHA256 CSR (CTRL + HASH0..7); instantiate once per fabric lane</t>
@@ -578,7 +578,7 @@
     <t>0x00000038</t>
   </si>
   <si>
-    <t>ID@0x0 magic[undefined:undefined] version[undefined:undefined]; STATUS@0x4 busy[undefined:undefined] code[undefined:undefined]; CFG@0x8 enable[undefined:undefined] mode[undefined:undefined]; FEED@0xc capture[undefined:undefined]; FIFO@0x10 data[undefined:undefined]; CMD@0x14 go[undefined:undefined]; IRQ@0x18 sticky[undefined:undefined]; BANK@0x1c cfg[undefined:undefined]; BANKSEL@0x2c bank_sel[undefined:undefined]; ACTIVE@0x34 value[undefined:undefined]; FABRIC@0x30 rb_grant_en[undefined:undefined]; key_key_0@0x20 key_0[undefined:undefined]; key_key_1@0x24 key_1[undefined:undefined]; key_key_2@0x28 key_2[undefined:undefined]</t>
+    <t>ID@0x0 magic[15:0] version[31:16]; STATUS@0x4 busy[0:0] code[15:8]; CFG@0x8 enable[0:0] mode[10:8]; FEED@0xc capture[15:0]; FIFO@0x10 data[31:0]; CMD@0x14 go[0:0]; IRQ@0x18 sticky[0:0]; BANK@0x1c cfg[7:0]; BANKSEL@0x2c bank_sel[1:0]; ACTIVE@0x34 value[7:0]; FABRIC@0x30 rb_grant_en[0:0]; key_key_0@0x20 key_0[31:0]; key_key_1@0x24 key_1[31:0]; key_key_2@0x28 key_2[31:0]</t>
   </si>
   <si>
     <t>SoC regfile smoke bank (RC/RO/RW/RWW/RWE/W1P/W1C/shadow/wide)</t>

</xml_diff>